<commit_message>
Add predicciones.xlsx of next 15 days
</commit_message>
<xml_diff>
--- a/p6_deployment/data/predicciones.xlsx
+++ b/p6_deployment/data/predicciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z4"/>
+  <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -567,227 +567,2377 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>80hEjzhl</t>
+          <t>hK8xvrmh</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45458.75</v>
+        <v>45462.97916666666</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>huracan</t>
+          <t>cf montreal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ind  rivadavia</t>
+          <t>new york red bulls</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>167</v>
       </c>
       <c r="F2" t="n">
-        <v>61</v>
+        <v>1671</v>
       </c>
       <c r="G2" t="n">
-        <v>1.67</v>
+        <v>3.25</v>
       </c>
       <c r="H2" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="I2" t="n">
-        <v>6</v>
+        <v>2.05</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5696460056964601</v>
+        <v>0.2866854423618529</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2718025227180252</v>
+        <v>0.2588132465766728</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1585514715855147</v>
+        <v>0.4545013110614742</v>
       </c>
       <c r="M2" t="n">
-        <v>0.05118334759053322</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+        <v>0.07327496351886609</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.2405712749555847</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.3047180572764508</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.4547106677679645</v>
+      </c>
       <c r="R2" t="n">
         <v>1</v>
       </c>
-      <c r="S2" t="inlineStr"/>
+      <c r="S2" t="n">
+        <v>0.0002093567064903601</v>
+      </c>
       <c r="T2" t="n">
-        <v>-100</v>
-      </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.0002093567064903601</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.4547106677679645</v>
+      </c>
       <c r="W2" t="n">
-        <v>1.30638852672751</v>
+        <v>2.05</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; 0.1</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y2" t="n">
+        <v>22.73553338839823</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>22.73553338839823</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>ChkVnhiD</t>
+          <t>rwisKhLu</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45458.85416666666</v>
+        <v>45462.97916666666</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>atl  tucuman</t>
+          <t>charlotte</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>defensa y justicia</t>
+          <t>orlando city</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>167</v>
       </c>
       <c r="F3" t="n">
-        <v>61</v>
+        <v>1671</v>
       </c>
       <c r="G3" t="n">
-        <v>1.91</v>
+        <v>2.05</v>
       </c>
       <c r="H3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I3" t="n">
         <v>3.4</v>
       </c>
-      <c r="I3" t="n">
-        <v>4.1</v>
-      </c>
       <c r="J3" t="n">
-        <v>0.4931894569255263</v>
+        <v>0.4603234298608499</v>
       </c>
       <c r="K3" t="n">
-        <v>0.2770564302140457</v>
+        <v>0.2621286197818729</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2297541128604281</v>
+        <v>0.2775479503572771</v>
       </c>
       <c r="M3" t="n">
-        <v>0.06158029550729749</v>
+        <v>0.05970030288538197</v>
       </c>
       <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.2991182851373308</v>
+        <v>0.2346391503667156</v>
       </c>
       <c r="P3" t="n">
-        <v>0.3871825052785184</v>
+        <v>0.3932230744752567</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3136992095841509</v>
+        <v>0.3721377751580278</v>
       </c>
       <c r="R3" t="n">
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1101260750644728</v>
+        <v>0.1310944546933838</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.1101260750644728</v>
+        <v>0.1310944546933838</v>
       </c>
       <c r="V3" t="n">
-        <v>0.3871825052785184</v>
+        <v>0.3932230744752567</v>
       </c>
       <c r="W3" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; 0.1</t>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>19.35912526392592</v>
+        <v>19.66115372376283</v>
       </c>
       <c r="Z3" t="n">
-        <v>19.35912526392592</v>
+        <v>19.66115372376283</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>UHaVQ4y2</t>
+          <t>2u7rIWkh</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45459.54166666666</v>
+        <v>45462.97916666666</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>river plate</t>
+          <t>dc united</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>talleres cordoba</t>
+          <t>atlanta utd</t>
         </is>
       </c>
       <c r="E4" t="n">
+        <v>167</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.4792284866468843</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.2459198813056379</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.2748516320474777</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.07009605461617863</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.3055089573397518</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.3831750237444987</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.3113160189157493</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.1372551424388608</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.1372551424388608</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.3831750237444987</v>
+      </c>
+      <c r="W4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y4" t="n">
+        <v>19.15875118722494</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>19.15875118722494</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>tW5nHj5b</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>45462.97916666666</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>inter miami</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>columbus crew</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>167</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.3461313584096667</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.2572597934125901</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.3966088481777431</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.05057330057330067</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.4505947056993999</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.4045720753855079</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.1448332189150922</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.1044633472897332</v>
+      </c>
+      <c r="T5" t="n">
+        <v>1</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.1044633472897332</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.4505947056993999</v>
+      </c>
+      <c r="W5" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y5" t="n">
+        <v>22.52973528496999</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>22.52973528496999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>WA7tw22b</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>45462.97916666666</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>toronto fc</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>nashville sc</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>167</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.4276704769412693</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.2688214426487978</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.303508080409933</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.06284038542103043</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.1818075392583132</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.3904373506291662</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.4277551101125207</v>
+      </c>
+      <c r="R6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.1242470297025876</v>
+      </c>
+      <c r="T6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.1242470297025876</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.4277551101125207</v>
+      </c>
+      <c r="W6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>21.38775550562603</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>21.38775550562603</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>MTkoJCzn</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>45462.98958333334</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fc cincinnati</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>philadelphia union</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>167</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.540711462450593</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.2490118577075099</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.2102766798418973</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.05680868838763553</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.4488093302829228</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.3709170360414691</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.1802736336756081</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="n">
+        <v>-0.09190213216767018</v>
+      </c>
+      <c r="T7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.09190213216767018</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.5511906697170772</v>
+      </c>
+      <c r="W7" t="n">
+        <v>2.060240963855422</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>27.55953348585386</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>27.55953348585386</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>zg5jGAK4</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>45463.02083333334</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>austin fc</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>los angeles fc</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>167</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.2690265486725664</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.2353982300884956</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.495575221238938</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.06203007518796988</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.1680032805977818</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.2809564326988208</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.5510402867033973</v>
+      </c>
+      <c r="R8" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.05546506546445928</v>
+      </c>
+      <c r="T8" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.05546506546445928</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.5510402867033973</v>
+      </c>
+      <c r="W8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>27.55201433516986</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>27.55201433516986</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>ld9fFUZA</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>45463.02083333334</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fc dallas</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>minnesota united</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>167</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.4569015166058744</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.2754847379535419</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.2676137454405835</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.06763681082188988</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.402282078998908</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.3889374590923115</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.2087804619087806</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="n">
+        <v>-0.05461943760696641</v>
+      </c>
+      <c r="T9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.05461943760696641</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.597717921001092</v>
+      </c>
+      <c r="W9" t="n">
+        <v>1.72463768115942</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>29.8858960500546</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>29.8858960500546</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>WKbaElkH</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>45463.02083333334</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>houston dynamo</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>seattle sounders</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>167</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="H10" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.4365343242714649</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.2607079992176805</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.3027576765108547</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.06547470200883554</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.400264628302527</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.3118599895825174</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.2878753821149555</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="n">
+        <v>-0.03626969596893787</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1</v>
+      </c>
+      <c r="U10" t="n">
+        <v>-0.03626969596893787</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0.400264628302527</v>
+      </c>
+      <c r="W10" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>20.01323141512635</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>20.01323141512635</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>ABc3D84N</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>45463.02083333334</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>sporting kansas city</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>real salt lake</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>167</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.3617021276595744</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.2765957446808511</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.3617021276595744</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.06334841628959276</v>
+      </c>
+      <c r="N11" t="n">
+        <v>2</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.3412578240487837</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.3137801616037382</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.3449620143474781</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="n">
+        <v>-0.01674011331209629</v>
+      </c>
+      <c r="T11" t="n">
+        <v>2</v>
+      </c>
+      <c r="U11" t="n">
+        <v>-0.01674011331209629</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0.3449620143474781</v>
+      </c>
+      <c r="W11" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>17.24810071737391</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>17.24810071737391</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>vo27CSJT</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45463.02083333334</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>st  louis city</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>colorado rapids</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>167</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.479807336050389</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.2528714338643941</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.2673212300852167</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.06880506880506898</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.5599963916364866</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.3240456798708019</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.1159579284927115</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.08018905558609762</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.08018905558609762</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.5599963916364866</v>
+      </c>
+      <c r="W12" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y12" t="n">
+        <v>27.99981958182433</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>27.99981958182433</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>tflZ7nSp</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45463.10416666666</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>los angeles galaxy</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>new york city</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>167</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.4697535474234503</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.2539208364451083</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.2763256161314414</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.06438791732909377</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.5002091728446787</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.3090900172899541</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.1907008098653671</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.03045562542122837</v>
+      </c>
+      <c r="T13" t="n">
+        <v>1</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.03045562542122837</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.5002091728446787</v>
+      </c>
+      <c r="W13" t="n">
+        <v>2</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y13" t="n">
+        <v>25.01045864223394</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>25.01045864223394</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>raSHWV4o</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45463.10416666666</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>san jose earthquakes</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>portland timbers</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>167</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4895104895104894</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.2447552447552447</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.2657342657342657</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.07518796992481214</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.3923500084565287</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.2800914764928201</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.3275585150506511</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>-0.09716048105396069</v>
+      </c>
+      <c r="T14" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.09716048105396069</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0.6076499915434712</v>
+      </c>
+      <c r="W14" t="n">
+        <v>1.821917808219178</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y14" t="n">
+        <v>30.38249957717356</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>30.38249957717356</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>z7pPU9Zc</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45465.97916666666</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>columbus crew</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>sporting kansas city</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>167</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.6861848124428179</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.192131747483989</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.1216834400731931</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.09573934837092724</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.408017959212156</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.4769070702407857</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.1150749705470585</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.2847753227567967</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.2847753227567967</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0.4769070702407857</v>
+      </c>
+      <c r="W15" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>23.84535351203928</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>23.84535351203928</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>EcqTTTl4</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>45465.97916666666</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>dc united</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>houston dynamo</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>167</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.3903891133319158</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.2698277695088242</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.3397831171592601</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.0900199323228108</v>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.4232775238390781</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.3253819680529937</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.2513405081079281</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0.03288841050716229</v>
+      </c>
+      <c r="T16" t="n">
+        <v>1</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.03288841050716229</v>
+      </c>
+      <c r="V16" t="n">
+        <v>0.4232775238390781</v>
+      </c>
+      <c r="W16" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y16" t="n">
+        <v>21.16387619195391</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>21.16387619195391</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>tpoLVkKi</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45465.97916666666</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>fc cincinnati</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>new england revolution</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>167</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I17" t="n">
         <v>6</v>
       </c>
-      <c r="F4" t="n">
-        <v>66</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
+      <c r="J17" t="n">
+        <v>0.6544202066590127</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.1928817451205511</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.1526980482204363</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.0914786967418546</v>
+      </c>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.4661798452488833</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.3456482867954284</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.1881718679556882</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>-0.1882403614101294</v>
+      </c>
+      <c r="T17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0.1882403614101294</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0.5338201547511168</v>
+      </c>
+      <c r="W17" t="n">
+        <v>2.651162790697675</v>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y17" t="n">
+        <v>26.69100773755584</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>26.69100773755584</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>ln2oxMH4</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45465.97916666666</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>new york red bulls</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>toronto fc</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>167</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="I18" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.6102841677943167</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.2232746955345061</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.1664411366711773</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.09238728750923864</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.4276350697450202</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.4631947153215034</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.1091702149334762</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" t="n">
+        <v>0.2399200197869973</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0.2399200197869973</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0.4631947153215034</v>
+      </c>
+      <c r="W18" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y18" t="n">
+        <v>23.15973576607517</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>23.15973576607517</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>WYwYSm4A</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>45465.97916666666</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>orlando city</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>chicago fire</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>167</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.5292352777002512</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.2474532514652525</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.2233114708344962</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.09220739137558542</v>
+      </c>
+      <c r="N19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.5176915657228428</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.3199702133278545</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.1623382209493025</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" t="n">
+        <v>-0.01154371197740844</v>
+      </c>
+      <c r="T19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U19" t="n">
+        <v>-0.01154371197740844</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0.5176915657228428</v>
+      </c>
+      <c r="W19" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y19" t="n">
+        <v>25.88457828614214</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>25.88457828614214</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>APxxS7JG</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>45465.97916666666</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>philadelphia union</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>charlotte</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>167</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I20" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.4992690880467783</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.2537951197571123</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.2469357921961093</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.09449613547974201</v>
+      </c>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.4304832510879221</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.3686093631115925</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.2009073858004855</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="n">
+        <v>-0.06878583695885626</v>
+      </c>
+      <c r="T20" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0.06878583695885626</v>
+      </c>
+      <c r="V20" t="n">
+        <v>0.5695167489120779</v>
+      </c>
+      <c r="W20" t="n">
+        <v>1.824657534246575</v>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y20" t="n">
+        <v>28.4758374456039</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>28.4758374456039</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>4nxtRRYM</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>45466.02083333334</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>minnesota united</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>austin fc</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>167</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I21" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.5102040816326531</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.2448979591836735</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.2448979591836735</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.0888888888888888</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.3435369954829963</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0.4667154373272834</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.1897475671897203</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.2218174781436099</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0.2218174781436099</v>
+      </c>
+      <c r="V21" t="n">
+        <v>0.4667154373272834</v>
+      </c>
+      <c r="W21" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y21" t="n">
+        <v>23.33577186636417</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>23.33577186636417</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>IktpQolT</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>45466.02083333334</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>nashville sc</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>new york city</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>167</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.3906945681211042</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.2764915405164737</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.3328138913624221</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.1128452867583303</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.4784893112705486</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.3135793977055996</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.2079312910238517</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.08779474314944435</v>
+      </c>
+      <c r="T22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0.08779474314944435</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0.4784893112705486</v>
+      </c>
+      <c r="W22" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y22" t="n">
+        <v>23.92446556352743</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>23.92446556352743</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>OWICL5dp</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>45466.02083333334</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>st  louis city</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>atlanta utd</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>167</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G23" t="n">
         <v>2</v>
       </c>
-      <c r="O4" t="n">
-        <v>0.4028577852796484</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.07065718925890503</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.5264850254614466</v>
-      </c>
-      <c r="R4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="n">
-        <v>-2</v>
-      </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="n">
-        <v>0.4735149745385534</v>
-      </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &lt; 0.1</t>
-        </is>
-      </c>
-      <c r="Y4" t="n">
-        <v>23.67574872692767</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>23.67574872692767</v>
+      <c r="H23" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.4585987261146497</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.2547770700636943</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.2866242038216561</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.09027777777777768</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.3774133555331881</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.3841034906612782</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.2384831538055338</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.1293264205975839</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0.1293264205975839</v>
+      </c>
+      <c r="V23" t="n">
+        <v>0.3841034906612782</v>
+      </c>
+      <c r="W23" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y23" t="n">
+        <v>19.20517453306391</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>19.20517453306391</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Sx1kytXA</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>45466.0625</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>colorado rapids</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>cf montreal</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>167</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="H24" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="I24" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.5523077419979976</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.2427247181938568</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.2049675398081457</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.08418251216864503</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.3526258454087228</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.371449036874041</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.2759251177172362</v>
+      </c>
+      <c r="R24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.1287243186801842</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0.1287243186801842</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0.371449036874041</v>
+      </c>
+      <c r="W24" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y24" t="n">
+        <v>18.57245184370205</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>18.57245184370205</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>2NHGKPBj</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>45466.0625</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>real salt lake</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>los angeles galaxy</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>167</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.5251641137855581</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.2450765864332604</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.2297592997811816</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.088095238095238</v>
+      </c>
+      <c r="N25" t="n">
+        <v>2</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.1954301815841236</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.3442148757946548</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.4603549426212216</v>
+      </c>
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0.2305956428400399</v>
+      </c>
+      <c r="T25" t="n">
+        <v>2</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0.2305956428400399</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0.4603549426212216</v>
+      </c>
+      <c r="W25" t="n">
+        <v>4</v>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y25" t="n">
+        <v>23.01774713106108</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>23.01774713106108</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>UT5bq9li</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>45466.10416666666</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>los angeles fc</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>san jose earthquakes</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>167</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H26" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="I26" t="n">
+        <v>9</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.7319778188539741</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.166358595194085</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.1016635859519408</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.09292929292929308</v>
+      </c>
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.4793928065542001</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.3185566013592205</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.2020505920865793</v>
+      </c>
+      <c r="R26" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" t="n">
+        <v>-0.2525850122997739</v>
+      </c>
+      <c r="T26" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U26" t="n">
+        <v>0.2525850122997739</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0.5206071934457999</v>
+      </c>
+      <c r="W26" t="n">
+        <v>3.413793103448276</v>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &lt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y26" t="n">
+        <v>26.03035967228999</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>26.03035967228999</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Ma0gz0nH</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>45466.10416666666</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>portland timbers</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>vancouver whitecaps</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>167</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H27" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.4093023255813953</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.2558139534883721</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.3348837209302326</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.08585858585858586</v>
+      </c>
+      <c r="N27" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.408009767301907</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.368000075623453</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.2239901570746398</v>
+      </c>
+      <c r="R27" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" t="n">
+        <v>-0.001292558279488321</v>
+      </c>
+      <c r="T27" t="n">
+        <v>1</v>
+      </c>
+      <c r="U27" t="n">
+        <v>-0.001292558279488321</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0.408009767301907</v>
+      </c>
+      <c r="W27" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y27" t="n">
+        <v>20.40048836509535</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>20.40048836509535</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>8K42rT3c</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>45466.10416666666</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>seattle sounders</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>fc dallas</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>167</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="H28" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I28" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.5508222068321281</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.2555203015026817</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.1936574916651903</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.08710648877683225</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.3538440300735814</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0.4160217396938514</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.2301342302325673</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0.1605014381911697</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0.1605014381911697</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0.4160217396938514</v>
+      </c>
+      <c r="W28" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
+        </is>
+      </c>
+      <c r="Y28" t="n">
+        <v>20.80108698469257</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>20.80108698469257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Determino si acerte o no la bet en update_results.py
</commit_message>
<xml_diff>
--- a/p6_deployment/data/predicciones.xlsx
+++ b/p6_deployment/data/predicciones.xlsx
@@ -429,10 +429,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC15"/>
+  <dimension ref="A1:AF15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id_match</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>date</t>
@@ -570,27 +575,42 @@
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>competition</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
           <t>result</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>acerte</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>z7pPU9Zc</t>
+          <t>Sx1kytXA</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.0625</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>columbus crew</t>
+          <t>colorado rapids</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>sporting kansas city</t>
+          <t>cf montreal</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -600,66 +620,66 @@
         <v>1671</v>
       </c>
       <c r="G2" t="n">
-        <v>1.48</v>
+        <v>1.45</v>
       </c>
       <c r="H2" t="n">
-        <v>4.5</v>
+        <v>4.75</v>
       </c>
       <c r="I2" t="n">
-        <v>6.25</v>
+        <v>6.5</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6386964914272737</v>
+        <v>0.6543046357615894</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2100601794027478</v>
+        <v>0.1997350993377483</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1512433291699784</v>
+        <v>0.1459602649006622</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0578978978978979</v>
+        <v>0.05402764204942079</v>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0.442947785562681</v>
+        <v>0.3128952493758644</v>
       </c>
       <c r="P2" t="n">
-        <v>0.3696567110004065</v>
+        <v>0.5361372692209605</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1873955034369123</v>
+        <v>0.150967481403175</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.1957487058645927</v>
+        <v>0.3364021698832122</v>
       </c>
       <c r="T2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1957487058645927</v>
+        <v>0.3364021698832122</v>
       </c>
       <c r="V2" t="n">
-        <v>0.557052214437319</v>
+        <v>0.5361372692209605</v>
       </c>
       <c r="W2" t="n">
-        <v>2.616279069767442</v>
+        <v>4.75</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.05</t>
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>38.99365501061233</v>
+        <v>37.52960884546724</v>
       </c>
       <c r="Z2" t="n">
-        <v>38.99365501061233</v>
+        <v>37.52960884546724</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -668,30 +688,43 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AC2" t="n">
-        <v>1</v>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>EcqTTTl4</t>
+          <t>2NHGKPBj</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45465.97916666666</v>
+        <v>45466.0625</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>dc united</t>
+          <t>real salt lake</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>houston dynamo</t>
+          <t>los angeles galaxy</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -701,55 +734,55 @@
         <v>1671</v>
       </c>
       <c r="G3" t="n">
-        <v>2.1</v>
+        <v>1.73</v>
       </c>
       <c r="H3" t="n">
-        <v>3.7</v>
+        <v>4.33</v>
       </c>
       <c r="I3" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="J3" t="n">
-        <v>0.449677174325864</v>
+        <v>0.54584017471928</v>
       </c>
       <c r="K3" t="n">
-        <v>0.2552221800227877</v>
+        <v>0.2180839497146315</v>
       </c>
       <c r="L3" t="n">
-        <v>0.2951006456513482</v>
+        <v>0.2360758755660886</v>
       </c>
       <c r="M3" t="n">
-        <v>0.05896074646074645</v>
+        <v>0.05898156429801493</v>
       </c>
       <c r="N3" t="n">
         <v>2</v>
       </c>
       <c r="O3" t="n">
-        <v>0.330849415970903</v>
+        <v>0.2957512568246276</v>
       </c>
       <c r="P3" t="n">
-        <v>0.2884875394026187</v>
+        <v>0.2512322781440824</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3806630446264782</v>
+        <v>0.4530164650312902</v>
       </c>
       <c r="R3" t="n">
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>0.08556239897512991</v>
+        <v>0.2169405894652016</v>
       </c>
       <c r="T3" t="n">
         <v>2</v>
       </c>
       <c r="U3" t="n">
-        <v>0.08556239897512991</v>
+        <v>0.2169405894652016</v>
       </c>
       <c r="V3" t="n">
-        <v>0.3806630446264782</v>
+        <v>0.4530164650312902</v>
       </c>
       <c r="W3" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -757,29 +790,42 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>26.64641312385347</v>
+        <v>31.71115255219031</v>
       </c>
       <c r="Z3" t="n">
-        <v>26.64641312385347</v>
+        <v>31.71115255219031</v>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="AC3" t="n">
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE3" t="n">
         <v>2</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>tpoLVkKi</t>
+          <t>z7pPU9Zc</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -787,12 +833,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>fc cincinnati</t>
+          <t>columbus crew</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>new england revolution</t>
+          <t>sporting kansas city</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -802,85 +848,98 @@
         <v>1671</v>
       </c>
       <c r="G4" t="n">
-        <v>1.55</v>
+        <v>1.38</v>
       </c>
       <c r="H4" t="n">
-        <v>4.33</v>
+        <v>5</v>
       </c>
       <c r="I4" t="n">
-        <v>5.5</v>
+        <v>7.5</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6098357297414951</v>
+        <v>0.6849315068493151</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2183014736949925</v>
+        <v>0.189041095890411</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1718627965635123</v>
+        <v>0.126027397260274</v>
       </c>
       <c r="M4" t="n">
-        <v>0.05792635435785254</v>
+        <v>0.05797101449275366</v>
       </c>
       <c r="N4" t="n">
         <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>0.5622116073024658</v>
+        <v>0.4761392615476333</v>
       </c>
       <c r="P4" t="n">
-        <v>0.3421246695652593</v>
+        <v>0.3071275721315585</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.09566372313227506</v>
+        <v>0.2167331663208083</v>
       </c>
       <c r="R4" t="n">
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>-0.04762412243902936</v>
+        <v>-0.2087922453016819</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.04762412243902936</v>
+        <v>-0.2087922453016819</v>
       </c>
       <c r="V4" t="n">
-        <v>0.5622116073024658</v>
+        <v>0.4761392615476333</v>
       </c>
       <c r="W4" t="n">
-        <v>1.55</v>
+        <v>1.38</v>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>39.3548125111726</v>
+        <v>33.32974830833433</v>
       </c>
       <c r="Z4" t="n">
-        <v>39.3548125111726</v>
+        <v>33.32974830833433</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AC4" t="n">
-        <v>2</v>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>ln2oxMH4</t>
+          <t>EcqTTTl4</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -888,12 +947,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>new york red bulls</t>
+          <t>dc united</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>toronto fc</t>
+          <t>houston dynamo</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -903,85 +962,98 @@
         <v>1671</v>
       </c>
       <c r="G5" t="n">
-        <v>1.62</v>
+        <v>2.2</v>
       </c>
       <c r="H5" t="n">
-        <v>4.33</v>
+        <v>3.7</v>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5888816959792844</v>
+        <v>0.4295665634674923</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2203206345234275</v>
+        <v>0.2554179566563468</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1907976694972882</v>
+        <v>0.315015479876161</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0482308328343739</v>
+        <v>0.05814905814905802</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4064097840638316</v>
+        <v>0.1700536136842038</v>
       </c>
       <c r="P5" t="n">
-        <v>0.406249628466087</v>
+        <v>0.4010800352937268</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.1873405874700815</v>
+        <v>0.4288663510220694</v>
       </c>
       <c r="R5" t="n">
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>-0.1824719119154528</v>
+        <v>0.1138508711459084</v>
       </c>
       <c r="T5" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="U5" t="n">
-        <v>0.1824719119154528</v>
+        <v>0.1138508711459084</v>
       </c>
       <c r="V5" t="n">
-        <v>0.5935902159361683</v>
+        <v>0.4288663510220694</v>
       </c>
       <c r="W5" t="n">
-        <v>2.320471596998928</v>
+        <v>3</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>41.55131511553179</v>
+        <v>30.02064457154486</v>
       </c>
       <c r="Z5" t="n">
-        <v>41.55131511553179</v>
+        <v>30.02064457154486</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AC5" t="n">
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>WYwYSm4A</t>
+          <t>tpoLVkKi</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -989,12 +1061,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>orlando city</t>
+          <t>fc cincinnati</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>chicago fire</t>
+          <t>new england revolution</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1004,70 +1076,70 @@
         <v>1671</v>
       </c>
       <c r="G6" t="n">
-        <v>1.73</v>
+        <v>1.6</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="I6" t="n">
-        <v>4.33</v>
+        <v>5</v>
       </c>
       <c r="J6" t="n">
-        <v>0.54584017471928</v>
+        <v>0.5968169761273209</v>
       </c>
       <c r="K6" t="n">
-        <v>0.2360758755660886</v>
+        <v>0.2122015915119363</v>
       </c>
       <c r="L6" t="n">
-        <v>0.2180839497146315</v>
+        <v>0.1909814323607427</v>
       </c>
       <c r="M6" t="n">
-        <v>0.05898156429801493</v>
+        <v>0.04722222222222228</v>
       </c>
       <c r="N6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>0.431972689407671</v>
+        <v>0.2399392096277449</v>
       </c>
       <c r="P6" t="n">
-        <v>0.3757237719572734</v>
+        <v>0.4835136265925929</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.1923035386350555</v>
+        <v>0.2765471637796623</v>
       </c>
       <c r="R6" t="n">
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.113867485311609</v>
+        <v>0.2713120350806566</v>
       </c>
       <c r="T6" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>0.113867485311609</v>
+        <v>0.2713120350806566</v>
       </c>
       <c r="V6" t="n">
-        <v>0.568027310592329</v>
+        <v>0.4835136265925929</v>
       </c>
       <c r="W6" t="n">
-        <v>2.079231692677071</v>
+        <v>4.5</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>39.76191174146303</v>
+        <v>33.8459538614815</v>
       </c>
       <c r="Z6" t="n">
-        <v>39.76191174146303</v>
+        <v>33.8459538614815</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -1075,14 +1147,27 @@
           <t>2</t>
         </is>
       </c>
-      <c r="AC6" t="n">
-        <v>1</v>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>APxxS7JG</t>
+          <t>ln2oxMH4</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -1090,12 +1175,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>philadelphia union</t>
+          <t>new york red bulls</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>charlotte</t>
+          <t>toronto fc</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1105,98 +1190,111 @@
         <v>1671</v>
       </c>
       <c r="G7" t="n">
-        <v>1.9</v>
+        <v>1.57</v>
       </c>
       <c r="H7" t="n">
-        <v>3.9</v>
+        <v>4.33</v>
       </c>
       <c r="I7" t="n">
-        <v>3.7</v>
+        <v>5.25</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4998268098372012</v>
+        <v>0.6018171661844011</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2435053688950468</v>
+        <v>0.2182108431661685</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2566678212677519</v>
+        <v>0.1799719906494304</v>
       </c>
       <c r="M7" t="n">
-        <v>0.05299631615421085</v>
+        <v>0.05836574785251614</v>
       </c>
       <c r="N7" t="n">
         <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>0.4352110096174183</v>
+        <v>0.4957472790711372</v>
       </c>
       <c r="P7" t="n">
-        <v>0.4322347323892172</v>
+        <v>0.2448591035222365</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.1325542579933644</v>
+        <v>0.2593936174066264</v>
       </c>
       <c r="R7" t="n">
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.06461580021978297</v>
+        <v>-0.1060698871132638</v>
       </c>
       <c r="T7" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="U7" t="n">
-        <v>0.06461580021978297</v>
+        <v>-0.1060698871132638</v>
       </c>
       <c r="V7" t="n">
-        <v>0.5647889903825818</v>
+        <v>0.4957472790711372</v>
       </c>
       <c r="W7" t="n">
-        <v>1.898684210526316</v>
+        <v>1.57</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>39.53522932678072</v>
+        <v>34.70230953497961</v>
       </c>
       <c r="Z7" t="n">
-        <v>39.53522932678072</v>
+        <v>34.70230953497961</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AC7" t="n">
-        <v>2</v>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>4nxtRRYM</t>
+          <t>WYwYSm4A</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45466.02083333334</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>minnesota united</t>
+          <t>orlando city</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>austin fc</t>
+          <t>chicago fire</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1206,98 +1304,111 @@
         <v>1671</v>
       </c>
       <c r="G8" t="n">
-        <v>1.73</v>
+        <v>1.65</v>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="I8" t="n">
-        <v>4.33</v>
+        <v>4.75</v>
       </c>
       <c r="J8" t="n">
-        <v>0.54584017471928</v>
+        <v>0.5746381507885073</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2360758755660886</v>
+        <v>0.225750702095485</v>
       </c>
       <c r="L8" t="n">
-        <v>0.2180839497146315</v>
+        <v>0.1996111471160078</v>
       </c>
       <c r="M8" t="n">
-        <v>0.05898156429801493</v>
+        <v>0.05468215994531778</v>
       </c>
       <c r="N8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>0.4585357639156413</v>
+        <v>0.2064575634094828</v>
       </c>
       <c r="P8" t="n">
-        <v>0.3362499079698303</v>
+        <v>0.4346844708020633</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.2052143281145281</v>
+        <v>0.3588579657884538</v>
       </c>
       <c r="R8" t="n">
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.08730441080363877</v>
+        <v>0.2089337687065784</v>
       </c>
       <c r="T8" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>0.08730441080363877</v>
+        <v>0.2089337687065784</v>
       </c>
       <c r="V8" t="n">
-        <v>0.5414642360843587</v>
+        <v>0.4346844708020633</v>
       </c>
       <c r="W8" t="n">
-        <v>2.079231692677071</v>
+        <v>4.2</v>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>37.90249652590511</v>
+        <v>30.42791295614444</v>
       </c>
       <c r="Z8" t="n">
-        <v>37.90249652590511</v>
+        <v>30.42791295614444</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC8" t="n">
-        <v>2</v>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>IktpQolT</t>
+          <t>APxxS7JG</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45466.02083333334</v>
+        <v>45465.97916666666</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>nashville sc</t>
+          <t>philadelphia union</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>new york city</t>
+          <t>charlotte</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1310,82 +1421,95 @@
         <v>2.25</v>
       </c>
       <c r="H9" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="I9" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="J9" t="n">
-        <v>0.4192972007147112</v>
+        <v>0.4194683346364347</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2858844550327576</v>
+        <v>0.2550820953870211</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2948183442525313</v>
+        <v>0.3254495699765442</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0599747474747474</v>
+        <v>0.05954230092161117</v>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" t="n">
-        <v>0.3762812603021553</v>
+        <v>0.1470755222311179</v>
       </c>
       <c r="P9" t="n">
-        <v>0.3362450625534014</v>
+        <v>0.3804223516987789</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2874736771444432</v>
+        <v>0.4725021260701033</v>
       </c>
       <c r="R9" t="n">
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.04301594041255591</v>
+        <v>0.1470525560935591</v>
       </c>
       <c r="T9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.04301594041255591</v>
+        <v>0.1470525560935591</v>
       </c>
       <c r="V9" t="n">
-        <v>0.3762812603021553</v>
+        <v>0.4725021260701033</v>
       </c>
       <c r="W9" t="n">
-        <v>2.25</v>
+        <v>2.9</v>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>26.33968822115087</v>
+        <v>33.07514882490723</v>
       </c>
       <c r="Z9" t="n">
-        <v>26.33968822115087</v>
+        <v>33.07514882490723</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AC9" t="n">
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>OWICL5dp</t>
+          <t>4nxtRRYM</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -1393,12 +1517,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>st  louis city</t>
+          <t>minnesota united</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>atlanta utd</t>
+          <t>austin fc</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1408,98 +1532,111 @@
         <v>1671</v>
       </c>
       <c r="G10" t="n">
-        <v>1.85</v>
+        <v>1.73</v>
       </c>
       <c r="H10" t="n">
         <v>4</v>
       </c>
       <c r="I10" t="n">
-        <v>3.8</v>
+        <v>4.33</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5129935875801552</v>
+        <v>0.54584017471928</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2372595342558218</v>
+        <v>0.2360758755660886</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2497468781640229</v>
+        <v>0.2180839497146315</v>
       </c>
       <c r="M10" t="n">
-        <v>0.05369843527738261</v>
+        <v>0.05898156429801493</v>
       </c>
       <c r="N10" t="n">
         <v>2</v>
       </c>
       <c r="O10" t="n">
-        <v>0.2433648073553128</v>
+        <v>0.3723226691402557</v>
       </c>
       <c r="P10" t="n">
-        <v>0.3403588267448442</v>
+        <v>0.1948158673714422</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4162763658998431</v>
+        <v>0.4328614634883022</v>
       </c>
       <c r="R10" t="n">
         <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>0.1665294877358202</v>
+        <v>0.2147775137736708</v>
       </c>
       <c r="T10" t="n">
         <v>2</v>
       </c>
       <c r="U10" t="n">
-        <v>0.1665294877358202</v>
+        <v>0.2147775137736708</v>
       </c>
       <c r="V10" t="n">
-        <v>0.4162763658998431</v>
+        <v>0.4328614634883022</v>
       </c>
       <c r="W10" t="n">
-        <v>3.8</v>
+        <v>4.33</v>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>29.13934561298902</v>
+        <v>30.30030244418116</v>
       </c>
       <c r="Z10" t="n">
-        <v>29.13934561298902</v>
+        <v>30.30030244418116</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC10" t="n">
-        <v>0</v>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Sx1kytXA</t>
+          <t>IktpQolT</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45466.0625</v>
+        <v>45466.02083333334</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>colorado rapids</t>
+          <t>nashville sc</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>cf montreal</t>
+          <t>new york city</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1509,98 +1646,111 @@
         <v>1671</v>
       </c>
       <c r="G11" t="n">
-        <v>1.45</v>
+        <v>2.63</v>
       </c>
       <c r="H11" t="n">
-        <v>4.75</v>
+        <v>3.5</v>
       </c>
       <c r="I11" t="n">
-        <v>6.5</v>
+        <v>2.6</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6543046357615894</v>
+        <v>0.3619297617627173</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1997350993377483</v>
+        <v>0.2719643638388418</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1459602649006622</v>
+        <v>0.3661058743984409</v>
       </c>
       <c r="M11" t="n">
-        <v>0.05402764204942079</v>
+        <v>0.05055780721179959</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0.3128952493758644</v>
+        <v>0.3328004140349778</v>
       </c>
       <c r="P11" t="n">
-        <v>0.5361372692209605</v>
+        <v>0.426784241468339</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.150967481403175</v>
+        <v>0.2404153444966831</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>0.3364021698832122</v>
+        <v>0.1548198776294972</v>
       </c>
       <c r="T11" t="n">
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>0.3364021698832122</v>
+        <v>0.1548198776294972</v>
       </c>
       <c r="V11" t="n">
-        <v>0.5361372692209605</v>
+        <v>0.426784241468339</v>
       </c>
       <c r="W11" t="n">
-        <v>4.75</v>
+        <v>3.5</v>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>37.52960884546724</v>
+        <v>29.87489690278373</v>
       </c>
       <c r="Z11" t="n">
-        <v>37.52960884546724</v>
+        <v>29.87489690278373</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC11" t="n">
-        <v>1</v>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>2NHGKPBj</t>
+          <t>OWICL5dp</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45466.0625</v>
+        <v>45466.02083333334</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>real salt lake</t>
+          <t>st  louis city</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>los angeles galaxy</t>
+          <t>atlanta utd</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1610,70 +1760,70 @@
         <v>1671</v>
       </c>
       <c r="G12" t="n">
-        <v>1.73</v>
+        <v>1.83</v>
       </c>
       <c r="H12" t="n">
-        <v>4.33</v>
+        <v>4.2</v>
       </c>
       <c r="I12" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="J12" t="n">
-        <v>0.54584017471928</v>
+        <v>0.5180518051805181</v>
       </c>
       <c r="K12" t="n">
-        <v>0.2180839497146315</v>
+        <v>0.2257225722572257</v>
       </c>
       <c r="L12" t="n">
-        <v>0.2360758755660886</v>
+        <v>0.2562256225622562</v>
       </c>
       <c r="M12" t="n">
-        <v>0.05898156429801493</v>
+        <v>0.05481359579720224</v>
       </c>
       <c r="N12" t="n">
         <v>2</v>
       </c>
       <c r="O12" t="n">
-        <v>0.2957512568246276</v>
+        <v>0.2032595674696957</v>
       </c>
       <c r="P12" t="n">
-        <v>0.2512322781440824</v>
+        <v>0.2226757413052</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.4530164650312902</v>
+        <v>0.5740646912251044</v>
       </c>
       <c r="R12" t="n">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2169405894652016</v>
+        <v>0.3178390686628482</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
       </c>
       <c r="U12" t="n">
-        <v>0.2169405894652016</v>
+        <v>0.3178390686628482</v>
       </c>
       <c r="V12" t="n">
-        <v>0.4530164650312902</v>
+        <v>0.5740646912251044</v>
       </c>
       <c r="W12" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>31.71115255219031</v>
+        <v>40.18452838575731</v>
       </c>
       <c r="Z12" t="n">
-        <v>31.71115255219031</v>
+        <v>40.18452838575731</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -1681,8 +1831,21 @@
           <t>1</t>
         </is>
       </c>
-      <c r="AC12" t="n">
-        <v>2</v>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1711,66 +1874,66 @@
         <v>1671</v>
       </c>
       <c r="G13" t="n">
-        <v>1.36</v>
+        <v>1.3</v>
       </c>
       <c r="H13" t="n">
-        <v>5.25</v>
+        <v>6.25</v>
       </c>
       <c r="I13" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="J13" t="n">
-        <v>0.6880733944954128</v>
+        <v>0.7239382239382238</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1782437745740498</v>
+        <v>0.1505791505791506</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1336828309305373</v>
+        <v>0.1254826254826255</v>
       </c>
       <c r="M13" t="n">
-        <v>0.06862745098039214</v>
+        <v>0.06256410256410261</v>
       </c>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>0.6288124535672187</v>
+        <v>0.3349990233680442</v>
       </c>
       <c r="P13" t="n">
-        <v>0.3013673527911105</v>
+        <v>0.3841275358129648</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.06982019364167102</v>
+        <v>0.280873440818991</v>
       </c>
       <c r="R13" t="n">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.05926094092819412</v>
+        <v>0.2335483852338142</v>
       </c>
       <c r="T13" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>0.05926094092819412</v>
+        <v>0.2335483852338142</v>
       </c>
       <c r="V13" t="n">
-        <v>0.3711875464327813</v>
+        <v>0.3841275358129648</v>
       </c>
       <c r="W13" t="n">
-        <v>3</v>
+        <v>6.25</v>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>25.98312825029469</v>
+        <v>26.88892750690754</v>
       </c>
       <c r="Z13" t="n">
-        <v>25.98312825029469</v>
+        <v>26.88892750690754</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -1782,8 +1945,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="AC13" t="n">
-        <v>1</v>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1833,45 +2009,45 @@
         <v>0.05796719450132803</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O14" t="n">
-        <v>0.5201066341798269</v>
+        <v>0.3153639087876114</v>
       </c>
       <c r="P14" t="n">
-        <v>0.4046451603515387</v>
+        <v>0.2454734549405155</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.07524820546863475</v>
+        <v>0.4391626362718731</v>
       </c>
       <c r="R14" t="n">
         <v>1</v>
       </c>
       <c r="S14" t="n">
-        <v>0.08047459125150191</v>
+        <v>0.1342565419828735</v>
       </c>
       <c r="T14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U14" t="n">
-        <v>0.08047459125150191</v>
+        <v>0.1342565419828735</v>
       </c>
       <c r="V14" t="n">
-        <v>0.5201066341798269</v>
+        <v>0.4391626362718731</v>
       </c>
       <c r="W14" t="n">
-        <v>2.15</v>
+        <v>3.1</v>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y14" t="n">
-        <v>36.40746439258788</v>
+        <v>30.74138453903112</v>
       </c>
       <c r="Z14" t="n">
-        <v>36.40746439258788</v>
+        <v>30.74138453903112</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -1883,8 +2059,21 @@
           <t>0</t>
         </is>
       </c>
-      <c r="AC14" t="n">
-        <v>1</v>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1913,79 +2102,92 @@
         <v>1671</v>
       </c>
       <c r="G15" t="n">
-        <v>1.45</v>
+        <v>1.57</v>
       </c>
       <c r="H15" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="I15" t="n">
-        <v>7</v>
+        <v>5.75</v>
       </c>
       <c r="J15" t="n">
-        <v>0.6538661131292164</v>
+        <v>0.6038755619308649</v>
       </c>
       <c r="K15" t="n">
-        <v>0.210690192008303</v>
+        <v>0.2312401542027946</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1354436948624805</v>
+        <v>0.1648842838663405</v>
       </c>
       <c r="M15" t="n">
-        <v>0.05473453749315826</v>
+        <v>0.05475815766188674</v>
       </c>
       <c r="N15" t="n">
+        <v>2</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.2068043869608158</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.242857704879984</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.5503379081592003</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.3854536242928598</v>
+      </c>
+      <c r="T15" t="n">
+        <v>2</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0.3854536242928598</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0.5503379081592003</v>
+      </c>
+      <c r="W15" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
+        </is>
+      </c>
+      <c r="Y15" t="n">
+        <v>38.52365357114402</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>38.52365357114402</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>MLS</t>
+        </is>
+      </c>
+      <c r="AE15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF15" t="n">
         <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0.3745130758574692</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0.4403573203792</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0.1851296037633309</v>
-      </c>
-      <c r="R15" t="n">
-        <v>1</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0.229667128370897</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0.229667128370897</v>
-      </c>
-      <c r="V15" t="n">
-        <v>0.4403573203792</v>
-      </c>
-      <c r="W15" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>dif_prob_mod_bm &gt; -0.05</t>
-        </is>
-      </c>
-      <c r="Y15" t="n">
-        <v>30.825012426544</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>30.825012426544</v>
-      </c>
-      <c r="AA15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AC15" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Pruebo dispatch de prueba
</commit_message>
<xml_diff>
--- a/p6_deployment/data/predicciones.xlsx
+++ b/p6_deployment/data/predicciones.xlsx
@@ -265,7 +265,7 @@
     <t>seattle sounders</t>
   </si>
   <si>
-    <t xml:space="preserve">fc dallas </t>
+    <t xml:space="preserve">fc dallas  </t>
   </si>
 </sst>
 </file>
@@ -275,7 +275,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -285,13 +285,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -352,16 +346,16 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -821,7 +815,7 @@
         <v>32</v>
       </c>
       <c r="B2" s="5">
-        <v>25568.875526226853</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>33</v>
@@ -919,7 +913,7 @@
         <v>40</v>
       </c>
       <c r="B3" s="5">
-        <v>25568.875526226853</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>41</v>
@@ -1017,7 +1011,7 @@
         <v>44</v>
       </c>
       <c r="B4" s="5">
-        <v>25568.875526215277</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>45</v>
@@ -1115,7 +1109,7 @@
         <v>48</v>
       </c>
       <c r="B5" s="5">
-        <v>25568.875526215277</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>49</v>
@@ -1213,7 +1207,7 @@
         <v>51</v>
       </c>
       <c r="B6" s="5">
-        <v>25568.875526215277</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>52</v>
@@ -1311,7 +1305,7 @@
         <v>55</v>
       </c>
       <c r="B7" s="5">
-        <v>25568.875526215277</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>56</v>
@@ -1409,7 +1403,7 @@
         <v>59</v>
       </c>
       <c r="B8" s="5">
-        <v>25568.875526215277</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>60</v>
@@ -1507,7 +1501,7 @@
         <v>62</v>
       </c>
       <c r="B9" s="5">
-        <v>25568.875526215277</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>63</v>
@@ -1605,7 +1599,7 @@
         <v>65</v>
       </c>
       <c r="B10" s="5">
-        <v>25568.875526226853</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>66</v>
@@ -1703,7 +1697,7 @@
         <v>68</v>
       </c>
       <c r="B11" s="5">
-        <v>25568.875526226853</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>69</v>
@@ -1801,7 +1795,7 @@
         <v>71</v>
       </c>
       <c r="B12" s="5">
-        <v>25568.875526226853</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>72</v>
@@ -1899,7 +1893,7 @@
         <v>74</v>
       </c>
       <c r="B13" s="5">
-        <v>25568.875526226853</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>75</v>
@@ -1997,7 +1991,7 @@
         <v>78</v>
       </c>
       <c r="B14" s="5">
-        <v>25568.875526226853</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>79</v>
@@ -2090,12 +2084,12 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="20.25">
       <c r="A15" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B15" s="5">
-        <v>25568.875526226853</v>
+        <v>25568.875520833335</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Genero dispatch de prueba
</commit_message>
<xml_diff>
--- a/p6_deployment/data/predicciones.xlsx
+++ b/p6_deployment/data/predicciones.xlsx
@@ -265,7 +265,7 @@
     <t>seattle sounders</t>
   </si>
   <si>
-    <t xml:space="preserve">fc dallas  </t>
+    <t xml:space="preserve">fc dallas   </t>
   </si>
 </sst>
 </file>
@@ -712,7 +712,7 @@
     <col min="32" max="32" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -810,7 +810,7 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
         <v>32</v>
       </c>
@@ -908,7 +908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
         <v>40</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
         <v>44</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
         <v>48</v>
       </c>
@@ -1202,7 +1202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1" t="s">
         <v>51</v>
       </c>
@@ -1300,7 +1300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1" t="s">
         <v>55</v>
       </c>
@@ -1398,7 +1398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1" t="s">
         <v>59</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1" t="s">
         <v>62</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1" t="s">
         <v>65</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1" t="s">
         <v>71</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1" t="s">
         <v>74</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1" t="s">
         <v>78</v>
       </c>

</xml_diff>

<commit_message>
Pruebo dispatch agregando filas a predicciones.xlsx
</commit_message>
<xml_diff>
--- a/p6_deployment/data/predicciones.xlsx
+++ b/p6_deployment/data/predicciones.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="89">
   <si>
     <t>id_match</t>
   </si>
@@ -257,6 +257,21 @@
   </si>
   <si>
     <t>vancouver whitecaps</t>
+  </si>
+  <si>
+    <t>aefejfasdfn</t>
+  </si>
+  <si>
+    <t>equipo1</t>
+  </si>
+  <si>
+    <t>equipo2</t>
+  </si>
+  <si>
+    <t>dsfivdfdiskv</t>
+  </si>
+  <si>
+    <t>AOKSDGA</t>
   </si>
   <si>
     <t>8K42rT3c</t>
@@ -332,7 +347,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -357,6 +372,9 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -675,41 +693,41 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AF15"/>
+  <dimension ref="A1:AF18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -2084,12 +2102,12 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
       <c r="A15" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B15" s="5">
-        <v>25568.875520833335</v>
+        <v>25568.375520833335</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>82</v>
@@ -2107,67 +2125,67 @@
         <v>1.57</v>
       </c>
       <c r="H15" s="8">
-        <v>4.1</v>
+        <v>1</v>
       </c>
       <c r="I15" s="8">
-        <v>5.75</v>
+        <v>2</v>
       </c>
       <c r="J15" s="8">
-        <v>0.6038755619308649</v>
+        <v>3</v>
       </c>
       <c r="K15" s="8">
-        <v>0.2312401542027946</v>
+        <v>0.2554618627826753</v>
       </c>
       <c r="L15" s="8">
-        <v>0.1648842838663405</v>
+        <v>0.3049060942889996</v>
       </c>
       <c r="M15" s="8">
-        <v>0.05475815766188674</v>
+        <v>0.05796719450132803</v>
       </c>
       <c r="N15" s="7">
         <v>2</v>
       </c>
       <c r="O15" s="8">
-        <v>0.2068043869608158</v>
+        <v>0.3153639087876114</v>
       </c>
       <c r="P15" s="8">
-        <v>0.242857704879984</v>
+        <v>0.2454734549405155</v>
       </c>
       <c r="Q15" s="8">
-        <v>0.5503379081592003</v>
+        <v>0.4391626362718731</v>
       </c>
       <c r="R15" s="7">
         <v>1</v>
       </c>
       <c r="S15" s="8">
-        <v>0.3854536242928598</v>
+        <v>0.1342565419828735</v>
       </c>
       <c r="T15" s="7">
         <v>2</v>
       </c>
       <c r="U15" s="8">
-        <v>0.3854536242928598</v>
+        <v>0.1342565419828735</v>
       </c>
       <c r="V15" s="8">
-        <v>0.5503379081592003</v>
+        <v>0.4391626362718731</v>
       </c>
       <c r="W15" s="8">
-        <v>5.75</v>
+        <v>3.1</v>
       </c>
       <c r="X15" s="6" t="s">
         <v>47</v>
       </c>
       <c r="Y15" s="8">
-        <v>38.52365357114402</v>
+        <v>30.74138453903112</v>
       </c>
       <c r="Z15" s="8">
-        <v>38.52365357114402</v>
-      </c>
-      <c r="AA15" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB15" s="6" t="s">
-        <v>54</v>
+        <v>30.74138453903112</v>
+      </c>
+      <c r="AA15" s="9">
+        <v>2</v>
+      </c>
+      <c r="AB15" s="9">
+        <v>0</v>
       </c>
       <c r="AC15" s="6" t="s">
         <v>38</v>
@@ -2179,6 +2197,300 @@
         <v>1</v>
       </c>
       <c r="AF15" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+      <c r="A16" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="5">
+        <v>25568.375520833335</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" s="7">
+        <v>167</v>
+      </c>
+      <c r="F16" s="7">
+        <v>1671</v>
+      </c>
+      <c r="G16" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="H16" s="8">
+        <v>1</v>
+      </c>
+      <c r="I16" s="8">
+        <v>2</v>
+      </c>
+      <c r="J16" s="8">
+        <v>3</v>
+      </c>
+      <c r="K16" s="8">
+        <v>0.2554618627826753</v>
+      </c>
+      <c r="L16" s="8">
+        <v>0.3049060942889996</v>
+      </c>
+      <c r="M16" s="8">
+        <v>0.05796719450132803</v>
+      </c>
+      <c r="N16" s="7">
+        <v>2</v>
+      </c>
+      <c r="O16" s="8">
+        <v>0.3153639087876114</v>
+      </c>
+      <c r="P16" s="8">
+        <v>0.2454734549405155</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="R16" s="7">
+        <v>1</v>
+      </c>
+      <c r="S16" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="T16" s="7">
+        <v>2</v>
+      </c>
+      <c r="U16" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="V16" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="W16" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="X16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y16" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="Z16" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="AA16" s="9">
+        <v>2</v>
+      </c>
+      <c r="AB16" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE16" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF16" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+      <c r="A17" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="5">
+        <v>25568.375520833335</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="7">
+        <v>167</v>
+      </c>
+      <c r="F17" s="7">
+        <v>1671</v>
+      </c>
+      <c r="G17" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="H17" s="8">
+        <v>1</v>
+      </c>
+      <c r="I17" s="8">
+        <v>2</v>
+      </c>
+      <c r="J17" s="8">
+        <v>3</v>
+      </c>
+      <c r="K17" s="8">
+        <v>0.2554618627826753</v>
+      </c>
+      <c r="L17" s="8">
+        <v>0.3049060942889996</v>
+      </c>
+      <c r="M17" s="8">
+        <v>0.05796719450132803</v>
+      </c>
+      <c r="N17" s="7">
+        <v>2</v>
+      </c>
+      <c r="O17" s="8">
+        <v>0.3153639087876114</v>
+      </c>
+      <c r="P17" s="8">
+        <v>0.2454734549405155</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="R17" s="7">
+        <v>1</v>
+      </c>
+      <c r="S17" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="T17" s="7">
+        <v>2</v>
+      </c>
+      <c r="U17" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="V17" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="W17" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="X17" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y17" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="Z17" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="AA17" s="9">
+        <v>2</v>
+      </c>
+      <c r="AB17" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD17" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE17" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF17" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="20.25">
+      <c r="A18" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="5">
+        <v>25568.875520833335</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E18" s="7">
+        <v>167</v>
+      </c>
+      <c r="F18" s="7">
+        <v>1671</v>
+      </c>
+      <c r="G18" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="H18" s="8">
+        <v>4.1</v>
+      </c>
+      <c r="I18" s="8">
+        <v>5.75</v>
+      </c>
+      <c r="J18" s="8">
+        <v>0.6038755619308649</v>
+      </c>
+      <c r="K18" s="8">
+        <v>0.2312401542027946</v>
+      </c>
+      <c r="L18" s="8">
+        <v>0.1648842838663405</v>
+      </c>
+      <c r="M18" s="8">
+        <v>0.05475815766188674</v>
+      </c>
+      <c r="N18" s="7">
+        <v>2</v>
+      </c>
+      <c r="O18" s="8">
+        <v>0.2068043869608158</v>
+      </c>
+      <c r="P18" s="8">
+        <v>0.242857704879984</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>0.5503379081592003</v>
+      </c>
+      <c r="R18" s="7">
+        <v>1</v>
+      </c>
+      <c r="S18" s="8">
+        <v>0.3854536242928598</v>
+      </c>
+      <c r="T18" s="7">
+        <v>2</v>
+      </c>
+      <c r="U18" s="8">
+        <v>0.3854536242928598</v>
+      </c>
+      <c r="V18" s="8">
+        <v>0.5503379081592003</v>
+      </c>
+      <c r="W18" s="8">
+        <v>5.75</v>
+      </c>
+      <c r="X18" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y18" s="8">
+        <v>38.52365357114402</v>
+      </c>
+      <c r="Z18" s="8">
+        <v>38.52365357114402</v>
+      </c>
+      <c r="AA18" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC18" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD18" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE18" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF18" s="7">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dispatch de prueba para confirmar el correcto funcionamiento de transfer.yml con environmental variables
</commit_message>
<xml_diff>
--- a/p6_deployment/data/predicciones.xlsx
+++ b/p6_deployment/data/predicciones.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="89">
   <si>
     <t>id_match</t>
   </si>
@@ -124,12 +124,6 @@
     <t>dif_prob_mod_bm &gt; -0.05</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>USA</t>
   </si>
   <si>
@@ -145,9 +139,6 @@
     <t>los angeles galaxy</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>z7pPU9Zc</t>
   </si>
   <si>
@@ -178,9 +169,6 @@
     <t>new england revolution</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>ln2oxMH4</t>
   </si>
   <si>
@@ -190,9 +178,6 @@
     <t>toronto fc</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>WYwYSm4A</t>
   </si>
   <si>
@@ -247,9 +232,6 @@
     <t>san jose earthquakes</t>
   </si>
   <si>
-    <t>6</t>
-  </si>
-  <si>
     <t>Ma0gz0nH</t>
   </si>
   <si>
@@ -272,6 +254,24 @@
   </si>
   <si>
     <t>AOKSDGA</t>
+  </si>
+  <si>
+    <t>AAAAAAAAA</t>
+  </si>
+  <si>
+    <t>jasdngdsagn</t>
+  </si>
+  <si>
+    <t>ejiq</t>
+  </si>
+  <si>
+    <t>BBBBBBBBBB</t>
+  </si>
+  <si>
+    <t>neoqirg</t>
+  </si>
+  <si>
+    <t>sjdnfsaj</t>
   </si>
   <si>
     <t>8K42rT3c</t>
@@ -290,7 +290,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -301,6 +301,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -347,7 +353,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -376,6 +382,12 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -390,6 +402,9 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -693,41 +708,41 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AF18"/>
+  <dimension ref="A1:AF20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -809,10 +824,10 @@
       <c r="Z1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="3" t="s">
         <v>27</v>
       </c>
       <c r="AC1" s="1" t="s">
@@ -907,17 +922,17 @@
       <c r="Z2" s="8">
         <v>37.52960884546724</v>
       </c>
-      <c r="AA2" s="6" t="s">
+      <c r="AA2" s="9">
+        <v>4</v>
+      </c>
+      <c r="AB2" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC2" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AB2" s="6" t="s">
+      <c r="AD2" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="AC2" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD2" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="AE2" s="7">
         <v>1</v>
@@ -928,16 +943,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B3" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E3" s="7">
         <v>167</v>
@@ -1005,17 +1020,17 @@
       <c r="Z3" s="8">
         <v>31.71115255219031</v>
       </c>
-      <c r="AA3" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB3" s="6" t="s">
+      <c r="AA3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD3" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="AC3" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD3" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="AE3" s="7">
         <v>2</v>
@@ -1026,16 +1041,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B4" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E4" s="7">
         <v>167</v>
@@ -1095,7 +1110,7 @@
         <v>1.38</v>
       </c>
       <c r="X4" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y4" s="8">
         <v>33.32974830833433</v>
@@ -1103,17 +1118,17 @@
       <c r="Z4" s="8">
         <v>33.32974830833433</v>
       </c>
-      <c r="AA4" s="6" t="s">
+      <c r="AA4" s="9">
+        <v>4</v>
+      </c>
+      <c r="AB4" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AB4" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="AC4" s="6" t="s">
-        <v>38</v>
-      </c>
       <c r="AD4" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE4" s="7">
         <v>1</v>
@@ -1124,16 +1139,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B5" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E5" s="7">
         <v>167</v>
@@ -1193,7 +1208,7 @@
         <v>3</v>
       </c>
       <c r="X5" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y5" s="8">
         <v>30.02064457154486</v>
@@ -1201,17 +1216,17 @@
       <c r="Z5" s="8">
         <v>30.02064457154486</v>
       </c>
-      <c r="AA5" s="6" t="s">
+      <c r="AA5" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="9">
+        <v>4</v>
+      </c>
+      <c r="AC5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD5" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="AB5" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="AC5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD5" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="AE5" s="7">
         <v>2</v>
@@ -1222,16 +1237,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B6" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E6" s="7">
         <v>167</v>
@@ -1291,7 +1306,7 @@
         <v>4.5</v>
       </c>
       <c r="X6" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y6" s="8">
         <v>33.8459538614815</v>
@@ -1299,17 +1314,17 @@
       <c r="Z6" s="8">
         <v>33.8459538614815</v>
       </c>
-      <c r="AA6" s="6" t="s">
+      <c r="AA6" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="9">
+        <v>2</v>
+      </c>
+      <c r="AC6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD6" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="AB6" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="AC6" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD6" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="AE6" s="7">
         <v>2</v>
@@ -1320,16 +1335,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B7" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E7" s="7">
         <v>167</v>
@@ -1389,7 +1404,7 @@
         <v>1.57</v>
       </c>
       <c r="X7" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y7" s="8">
         <v>34.70230953497961</v>
@@ -1397,17 +1412,17 @@
       <c r="Z7" s="8">
         <v>34.70230953497961</v>
       </c>
-      <c r="AA7" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB7" s="6" t="s">
-        <v>43</v>
+      <c r="AA7" s="9">
+        <v>3</v>
+      </c>
+      <c r="AB7" s="9">
+        <v>0</v>
       </c>
       <c r="AC7" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AD7" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE7" s="7">
         <v>1</v>
@@ -1418,16 +1433,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B8" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E8" s="7">
         <v>167</v>
@@ -1487,7 +1502,7 @@
         <v>4.2</v>
       </c>
       <c r="X8" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y8" s="8">
         <v>30.42791295614444</v>
@@ -1495,17 +1510,17 @@
       <c r="Z8" s="8">
         <v>30.42791295614444</v>
       </c>
-      <c r="AA8" s="6" t="s">
+      <c r="AA8" s="9">
+        <v>4</v>
+      </c>
+      <c r="AB8" s="9">
+        <v>2</v>
+      </c>
+      <c r="AC8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AB8" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="AC8" s="6" t="s">
-        <v>38</v>
-      </c>
       <c r="AD8" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE8" s="7">
         <v>1</v>
@@ -1516,16 +1531,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B9" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E9" s="7">
         <v>167</v>
@@ -1585,7 +1600,7 @@
         <v>2.9</v>
       </c>
       <c r="X9" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y9" s="8">
         <v>33.07514882490723</v>
@@ -1593,17 +1608,17 @@
       <c r="Z9" s="8">
         <v>33.07514882490723</v>
       </c>
-      <c r="AA9" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB9" s="6" t="s">
-        <v>54</v>
+      <c r="AA9" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="9">
+        <v>2</v>
       </c>
       <c r="AC9" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AD9" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE9" s="7">
         <v>2</v>
@@ -1614,16 +1629,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B10" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E10" s="7">
         <v>167</v>
@@ -1683,7 +1698,7 @@
         <v>4.33</v>
       </c>
       <c r="X10" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y10" s="8">
         <v>30.30030244418116</v>
@@ -1691,17 +1706,17 @@
       <c r="Z10" s="8">
         <v>30.30030244418116</v>
       </c>
-      <c r="AA10" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB10" s="6" t="s">
+      <c r="AA10" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD10" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="AC10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD10" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="AE10" s="7">
         <v>2</v>
@@ -1712,16 +1727,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B11" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E11" s="7">
         <v>167</v>
@@ -1781,7 +1796,7 @@
         <v>3.5</v>
       </c>
       <c r="X11" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y11" s="8">
         <v>29.87489690278373</v>
@@ -1789,17 +1804,17 @@
       <c r="Z11" s="8">
         <v>29.87489690278373</v>
       </c>
-      <c r="AA11" s="6" t="s">
+      <c r="AA11" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB11" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD11" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="AB11" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="AC11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD11" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="AE11" s="7">
         <v>1</v>
@@ -1810,16 +1825,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B12" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E12" s="7">
         <v>167</v>
@@ -1879,7 +1894,7 @@
         <v>3.7</v>
       </c>
       <c r="X12" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y12" s="8">
         <v>40.18452838575731</v>
@@ -1887,17 +1902,17 @@
       <c r="Z12" s="8">
         <v>40.18452838575731</v>
       </c>
-      <c r="AA12" s="6" t="s">
+      <c r="AA12" s="9">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="9">
+        <v>1</v>
+      </c>
+      <c r="AC12" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD12" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="AB12" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="AC12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD12" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="AE12" s="7">
         <v>0</v>
@@ -1908,16 +1923,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B13" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E13" s="7">
         <v>167</v>
@@ -1977,7 +1992,7 @@
         <v>6.25</v>
       </c>
       <c r="X13" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y13" s="8">
         <v>26.88892750690754</v>
@@ -1985,17 +2000,17 @@
       <c r="Z13" s="8">
         <v>26.88892750690754</v>
       </c>
-      <c r="AA13" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="AB13" s="6" t="s">
-        <v>54</v>
+      <c r="AA13" s="9">
+        <v>6</v>
+      </c>
+      <c r="AB13" s="9">
+        <v>2</v>
       </c>
       <c r="AC13" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AD13" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE13" s="7">
         <v>1</v>
@@ -2006,16 +2021,16 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B14" s="5">
         <v>25568.875520833335</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E14" s="7">
         <v>167</v>
@@ -2075,7 +2090,7 @@
         <v>3.1</v>
       </c>
       <c r="X14" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y14" s="8">
         <v>30.74138453903112</v>
@@ -2083,17 +2098,17 @@
       <c r="Z14" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA14" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="AB14" s="6" t="s">
-        <v>43</v>
+      <c r="AA14" s="9">
+        <v>2</v>
+      </c>
+      <c r="AB14" s="9">
+        <v>0</v>
       </c>
       <c r="AC14" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AD14" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE14" s="7">
         <v>1</v>
@@ -2102,18 +2117,18 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B15" s="5">
         <v>25568.375520833335</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E15" s="7">
         <v>167</v>
@@ -2173,7 +2188,7 @@
         <v>3.1</v>
       </c>
       <c r="X15" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y15" s="8">
         <v>30.74138453903112</v>
@@ -2181,17 +2196,17 @@
       <c r="Z15" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA15" s="9">
-        <v>2</v>
-      </c>
-      <c r="AB15" s="9">
+      <c r="AA15" s="10">
+        <v>2</v>
+      </c>
+      <c r="AB15" s="10">
         <v>0</v>
       </c>
       <c r="AC15" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AD15" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE15" s="7">
         <v>1</v>
@@ -2200,18 +2215,18 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="1" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B16" s="5">
         <v>25568.375520833335</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E16" s="7">
         <v>167</v>
@@ -2271,7 +2286,7 @@
         <v>3.1</v>
       </c>
       <c r="X16" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y16" s="8">
         <v>30.74138453903112</v>
@@ -2279,17 +2294,17 @@
       <c r="Z16" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA16" s="9">
-        <v>2</v>
-      </c>
-      <c r="AB16" s="9">
+      <c r="AA16" s="10">
+        <v>2</v>
+      </c>
+      <c r="AB16" s="10">
         <v>0</v>
       </c>
       <c r="AC16" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AD16" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE16" s="7">
         <v>1</v>
@@ -2298,18 +2313,18 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B17" s="5">
         <v>25568.375520833335</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E17" s="7">
         <v>167</v>
@@ -2369,7 +2384,7 @@
         <v>3.1</v>
       </c>
       <c r="X17" s="6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Y17" s="8">
         <v>30.74138453903112</v>
@@ -2377,17 +2392,17 @@
       <c r="Z17" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA17" s="9">
-        <v>2</v>
-      </c>
-      <c r="AB17" s="9">
+      <c r="AA17" s="10">
+        <v>2</v>
+      </c>
+      <c r="AB17" s="10">
         <v>0</v>
       </c>
       <c r="AC17" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AD17" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AE17" s="7">
         <v>1</v>
@@ -2396,18 +2411,18 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="20.25">
-      <c r="A18" s="1" t="s">
-        <v>86</v>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
+      <c r="A18" s="11" t="s">
+        <v>80</v>
       </c>
       <c r="B18" s="5">
-        <v>25568.875520833335</v>
+        <v>25568.375520833335</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E18" s="7">
         <v>167</v>
@@ -2419,78 +2434,274 @@
         <v>1.57</v>
       </c>
       <c r="H18" s="8">
+        <v>1</v>
+      </c>
+      <c r="I18" s="8">
+        <v>2</v>
+      </c>
+      <c r="J18" s="8">
+        <v>3</v>
+      </c>
+      <c r="K18" s="8">
+        <v>0.2554618627826753</v>
+      </c>
+      <c r="L18" s="8">
+        <v>0.3049060942889996</v>
+      </c>
+      <c r="M18" s="8">
+        <v>0.05796719450132803</v>
+      </c>
+      <c r="N18" s="7">
+        <v>2</v>
+      </c>
+      <c r="O18" s="8">
+        <v>0.3153639087876114</v>
+      </c>
+      <c r="P18" s="8">
+        <v>0.2454734549405155</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="R18" s="7">
+        <v>1</v>
+      </c>
+      <c r="S18" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="T18" s="7">
+        <v>2</v>
+      </c>
+      <c r="U18" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="V18" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="W18" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="X18" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y18" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="Z18" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="AA18" s="10">
+        <v>2</v>
+      </c>
+      <c r="AB18" s="10">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD18" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE18" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF18" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+      <c r="A19" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" s="5">
+        <v>25568.375520833335</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E19" s="7">
+        <v>167</v>
+      </c>
+      <c r="F19" s="7">
+        <v>1671</v>
+      </c>
+      <c r="G19" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="H19" s="8">
+        <v>1</v>
+      </c>
+      <c r="I19" s="8">
+        <v>2</v>
+      </c>
+      <c r="J19" s="8">
+        <v>3</v>
+      </c>
+      <c r="K19" s="8">
+        <v>0.2554618627826753</v>
+      </c>
+      <c r="L19" s="8">
+        <v>0.3049060942889996</v>
+      </c>
+      <c r="M19" s="8">
+        <v>0.05796719450132803</v>
+      </c>
+      <c r="N19" s="7">
+        <v>2</v>
+      </c>
+      <c r="O19" s="8">
+        <v>0.3153639087876114</v>
+      </c>
+      <c r="P19" s="8">
+        <v>0.2454734549405155</v>
+      </c>
+      <c r="Q19" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="R19" s="7">
+        <v>1</v>
+      </c>
+      <c r="S19" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="T19" s="7">
+        <v>2</v>
+      </c>
+      <c r="U19" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="V19" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="W19" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="X19" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y19" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="Z19" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="AA19" s="10">
+        <v>2</v>
+      </c>
+      <c r="AB19" s="10">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD19" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE19" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF19" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="20.25">
+      <c r="A20" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" s="5">
+        <v>25568.875520833335</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E20" s="7">
+        <v>167</v>
+      </c>
+      <c r="F20" s="7">
+        <v>1671</v>
+      </c>
+      <c r="G20" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="H20" s="8">
         <v>4.1</v>
       </c>
-      <c r="I18" s="8">
+      <c r="I20" s="8">
         <v>5.75</v>
       </c>
-      <c r="J18" s="8">
+      <c r="J20" s="8">
         <v>0.6038755619308649</v>
       </c>
-      <c r="K18" s="8">
+      <c r="K20" s="8">
         <v>0.2312401542027946</v>
       </c>
-      <c r="L18" s="8">
+      <c r="L20" s="8">
         <v>0.1648842838663405</v>
       </c>
-      <c r="M18" s="8">
+      <c r="M20" s="8">
         <v>0.05475815766188674</v>
       </c>
-      <c r="N18" s="7">
-        <v>2</v>
-      </c>
-      <c r="O18" s="8">
+      <c r="N20" s="7">
+        <v>2</v>
+      </c>
+      <c r="O20" s="8">
         <v>0.2068043869608158</v>
       </c>
-      <c r="P18" s="8">
+      <c r="P20" s="8">
         <v>0.242857704879984</v>
       </c>
-      <c r="Q18" s="8">
+      <c r="Q20" s="8">
         <v>0.5503379081592003</v>
       </c>
-      <c r="R18" s="7">
-        <v>1</v>
-      </c>
-      <c r="S18" s="8">
+      <c r="R20" s="7">
+        <v>1</v>
+      </c>
+      <c r="S20" s="8">
         <v>0.3854536242928598</v>
       </c>
-      <c r="T18" s="7">
-        <v>2</v>
-      </c>
-      <c r="U18" s="8">
+      <c r="T20" s="7">
+        <v>2</v>
+      </c>
+      <c r="U20" s="8">
         <v>0.3854536242928598</v>
       </c>
-      <c r="V18" s="8">
+      <c r="V20" s="8">
         <v>0.5503379081592003</v>
       </c>
-      <c r="W18" s="8">
+      <c r="W20" s="8">
         <v>5.75</v>
       </c>
-      <c r="X18" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y18" s="8">
+      <c r="X20" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y20" s="8">
         <v>38.52365357114402</v>
       </c>
-      <c r="Z18" s="8">
+      <c r="Z20" s="8">
         <v>38.52365357114402</v>
       </c>
-      <c r="AA18" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="AB18" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="AC18" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="AD18" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE18" s="7">
-        <v>1</v>
-      </c>
-      <c r="AF18" s="7">
+      <c r="AA20" s="9">
+        <v>3</v>
+      </c>
+      <c r="AB20" s="9">
+        <v>2</v>
+      </c>
+      <c r="AC20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD20" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE20" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF20" s="7">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ultima prueba de transfer.yml con environmental variables
</commit_message>
<xml_diff>
--- a/p6_deployment/data/predicciones.xlsx
+++ b/p6_deployment/data/predicciones.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="90">
   <si>
     <t>id_match</t>
   </si>
@@ -272,6 +272,9 @@
   </si>
   <si>
     <t>sjdnfsaj</t>
+  </si>
+  <si>
+    <t>ZZZZZZZZ</t>
   </si>
   <si>
     <t>8K42rT3c</t>
@@ -353,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -379,11 +382,11 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -402,9 +405,6 @@
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -708,7 +708,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AF20"/>
+  <dimension ref="A1:AF21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
@@ -737,8 +737,8 @@
     <col min="24" max="24" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="25" max="25" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="26" max="26" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="29" max="29" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="30" max="30" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="31" max="31" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
@@ -2196,10 +2196,10 @@
       <c r="Z15" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA15" s="10">
-        <v>2</v>
-      </c>
-      <c r="AB15" s="10">
+      <c r="AA15" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB15" s="7">
         <v>0</v>
       </c>
       <c r="AC15" s="6" t="s">
@@ -2294,10 +2294,10 @@
       <c r="Z16" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA16" s="10">
-        <v>2</v>
-      </c>
-      <c r="AB16" s="10">
+      <c r="AA16" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB16" s="7">
         <v>0</v>
       </c>
       <c r="AC16" s="6" t="s">
@@ -2313,7 +2313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="20.25">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
@@ -2392,10 +2392,10 @@
       <c r="Z17" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA17" s="10">
-        <v>2</v>
-      </c>
-      <c r="AB17" s="10">
+      <c r="AA17" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB17" s="7">
         <v>0</v>
       </c>
       <c r="AC17" s="6" t="s">
@@ -2411,8 +2411,8 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="17.25">
-      <c r="A18" s="11" t="s">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+      <c r="A18" s="10" t="s">
         <v>80</v>
       </c>
       <c r="B18" s="5">
@@ -2490,10 +2490,10 @@
       <c r="Z18" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA18" s="10">
-        <v>2</v>
-      </c>
-      <c r="AB18" s="10">
+      <c r="AA18" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB18" s="7">
         <v>0</v>
       </c>
       <c r="AC18" s="6" t="s">
@@ -2509,8 +2509,8 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
-      <c r="A19" s="11" t="s">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
+      <c r="A19" s="10" t="s">
         <v>83</v>
       </c>
       <c r="B19" s="5">
@@ -2588,10 +2588,10 @@
       <c r="Z19" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA19" s="10">
-        <v>2</v>
-      </c>
-      <c r="AB19" s="10">
+      <c r="AA19" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB19" s="7">
         <v>0</v>
       </c>
       <c r="AC19" s="6" t="s">
@@ -2607,18 +2607,18 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="20.25">
-      <c r="A20" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
+      <c r="A20" s="11" t="s">
         <v>86</v>
       </c>
       <c r="B20" s="5">
-        <v>25568.875520833335</v>
+        <v>25568.375520833335</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E20" s="7">
         <v>167</v>
@@ -2630,67 +2630,67 @@
         <v>1.57</v>
       </c>
       <c r="H20" s="8">
-        <v>4.1</v>
+        <v>1</v>
       </c>
       <c r="I20" s="8">
-        <v>5.75</v>
+        <v>2</v>
       </c>
       <c r="J20" s="8">
-        <v>0.6038755619308649</v>
+        <v>3</v>
       </c>
       <c r="K20" s="8">
-        <v>0.2312401542027946</v>
+        <v>0.2554618627826753</v>
       </c>
       <c r="L20" s="8">
-        <v>0.1648842838663405</v>
+        <v>0.3049060942889996</v>
       </c>
       <c r="M20" s="8">
-        <v>0.05475815766188674</v>
+        <v>0.05796719450132803</v>
       </c>
       <c r="N20" s="7">
         <v>2</v>
       </c>
       <c r="O20" s="8">
-        <v>0.2068043869608158</v>
+        <v>0.3153639087876114</v>
       </c>
       <c r="P20" s="8">
-        <v>0.242857704879984</v>
+        <v>0.2454734549405155</v>
       </c>
       <c r="Q20" s="8">
-        <v>0.5503379081592003</v>
+        <v>0.4391626362718731</v>
       </c>
       <c r="R20" s="7">
         <v>1</v>
       </c>
       <c r="S20" s="8">
-        <v>0.3854536242928598</v>
+        <v>0.1342565419828735</v>
       </c>
       <c r="T20" s="7">
         <v>2</v>
       </c>
       <c r="U20" s="8">
-        <v>0.3854536242928598</v>
+        <v>0.1342565419828735</v>
       </c>
       <c r="V20" s="8">
-        <v>0.5503379081592003</v>
+        <v>0.4391626362718731</v>
       </c>
       <c r="W20" s="8">
-        <v>5.75</v>
+        <v>3.1</v>
       </c>
       <c r="X20" s="6" t="s">
         <v>44</v>
       </c>
       <c r="Y20" s="8">
-        <v>38.52365357114402</v>
+        <v>30.74138453903112</v>
       </c>
       <c r="Z20" s="8">
-        <v>38.52365357114402</v>
-      </c>
-      <c r="AA20" s="9">
-        <v>3</v>
-      </c>
-      <c r="AB20" s="9">
-        <v>2</v>
+        <v>30.74138453903112</v>
+      </c>
+      <c r="AA20" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB20" s="7">
+        <v>0</v>
       </c>
       <c r="AC20" s="6" t="s">
         <v>36</v>
@@ -2702,6 +2702,104 @@
         <v>1</v>
       </c>
       <c r="AF20" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="20.25">
+      <c r="A21" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="5">
+        <v>25568.875520833335</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E21" s="7">
+        <v>167</v>
+      </c>
+      <c r="F21" s="7">
+        <v>1671</v>
+      </c>
+      <c r="G21" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="H21" s="8">
+        <v>4.1</v>
+      </c>
+      <c r="I21" s="8">
+        <v>5.75</v>
+      </c>
+      <c r="J21" s="8">
+        <v>0.6038755619308649</v>
+      </c>
+      <c r="K21" s="8">
+        <v>0.2312401542027946</v>
+      </c>
+      <c r="L21" s="8">
+        <v>0.1648842838663405</v>
+      </c>
+      <c r="M21" s="8">
+        <v>0.05475815766188674</v>
+      </c>
+      <c r="N21" s="7">
+        <v>2</v>
+      </c>
+      <c r="O21" s="8">
+        <v>0.2068043869608158</v>
+      </c>
+      <c r="P21" s="8">
+        <v>0.242857704879984</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>0.5503379081592003</v>
+      </c>
+      <c r="R21" s="7">
+        <v>1</v>
+      </c>
+      <c r="S21" s="8">
+        <v>0.3854536242928598</v>
+      </c>
+      <c r="T21" s="7">
+        <v>2</v>
+      </c>
+      <c r="U21" s="8">
+        <v>0.3854536242928598</v>
+      </c>
+      <c r="V21" s="8">
+        <v>0.5503379081592003</v>
+      </c>
+      <c r="W21" s="8">
+        <v>5.75</v>
+      </c>
+      <c r="X21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y21" s="8">
+        <v>38.52365357114402</v>
+      </c>
+      <c r="Z21" s="8">
+        <v>38.52365357114402</v>
+      </c>
+      <c r="AA21" s="9">
+        <v>3</v>
+      </c>
+      <c r="AB21" s="9">
+        <v>2</v>
+      </c>
+      <c r="AC21" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD21" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE21" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF21" s="7">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrego dos filas artificiales mas
</commit_message>
<xml_diff>
--- a/p6_deployment/data/predicciones.xlsx
+++ b/p6_deployment/data/predicciones.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="92">
   <si>
     <t>id_match</t>
   </si>
@@ -274,7 +274,13 @@
     <t>sjdnfsaj</t>
   </si>
   <si>
+    <t>XXXXXXXXXX</t>
+  </si>
+  <si>
     <t>ZZZZZZZZ</t>
+  </si>
+  <si>
+    <t>nueva_fila</t>
   </si>
   <si>
     <t>8K42rT3c</t>
@@ -382,13 +388,13 @@
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -708,7 +714,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AF21"/>
+  <dimension ref="A1:AF23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
@@ -922,10 +928,10 @@
       <c r="Z2" s="8">
         <v>37.52960884546724</v>
       </c>
-      <c r="AA2" s="9">
+      <c r="AA2" s="7">
         <v>4</v>
       </c>
-      <c r="AB2" s="9">
+      <c r="AB2" s="7">
         <v>1</v>
       </c>
       <c r="AC2" s="6" t="s">
@@ -1020,10 +1026,10 @@
       <c r="Z3" s="8">
         <v>31.71115255219031</v>
       </c>
-      <c r="AA3" s="9">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="9">
+      <c r="AA3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="7">
         <v>1</v>
       </c>
       <c r="AC3" s="6" t="s">
@@ -1118,10 +1124,10 @@
       <c r="Z4" s="8">
         <v>33.32974830833433</v>
       </c>
-      <c r="AA4" s="9">
+      <c r="AA4" s="7">
         <v>4</v>
       </c>
-      <c r="AB4" s="9">
+      <c r="AB4" s="7">
         <v>0</v>
       </c>
       <c r="AC4" s="6" t="s">
@@ -1216,10 +1222,10 @@
       <c r="Z5" s="8">
         <v>30.02064457154486</v>
       </c>
-      <c r="AA5" s="9">
-        <v>1</v>
-      </c>
-      <c r="AB5" s="9">
+      <c r="AA5" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="7">
         <v>4</v>
       </c>
       <c r="AC5" s="6" t="s">
@@ -1314,10 +1320,10 @@
       <c r="Z6" s="8">
         <v>33.8459538614815</v>
       </c>
-      <c r="AA6" s="9">
-        <v>1</v>
-      </c>
-      <c r="AB6" s="9">
+      <c r="AA6" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="7">
         <v>2</v>
       </c>
       <c r="AC6" s="6" t="s">
@@ -1412,10 +1418,10 @@
       <c r="Z7" s="8">
         <v>34.70230953497961</v>
       </c>
-      <c r="AA7" s="9">
+      <c r="AA7" s="7">
         <v>3</v>
       </c>
-      <c r="AB7" s="9">
+      <c r="AB7" s="7">
         <v>0</v>
       </c>
       <c r="AC7" s="6" t="s">
@@ -1510,10 +1516,10 @@
       <c r="Z8" s="8">
         <v>30.42791295614444</v>
       </c>
-      <c r="AA8" s="9">
+      <c r="AA8" s="7">
         <v>4</v>
       </c>
-      <c r="AB8" s="9">
+      <c r="AB8" s="7">
         <v>2</v>
       </c>
       <c r="AC8" s="6" t="s">
@@ -1608,10 +1614,10 @@
       <c r="Z9" s="8">
         <v>33.07514882490723</v>
       </c>
-      <c r="AA9" s="9">
-        <v>0</v>
-      </c>
-      <c r="AB9" s="9">
+      <c r="AA9" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="7">
         <v>2</v>
       </c>
       <c r="AC9" s="6" t="s">
@@ -1706,10 +1712,10 @@
       <c r="Z10" s="8">
         <v>30.30030244418116</v>
       </c>
-      <c r="AA10" s="9">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="9">
+      <c r="AA10" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="7">
         <v>1</v>
       </c>
       <c r="AC10" s="6" t="s">
@@ -1804,10 +1810,10 @@
       <c r="Z11" s="8">
         <v>29.87489690278373</v>
       </c>
-      <c r="AA11" s="9">
-        <v>1</v>
-      </c>
-      <c r="AB11" s="9">
+      <c r="AA11" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB11" s="7">
         <v>0</v>
       </c>
       <c r="AC11" s="6" t="s">
@@ -1902,10 +1908,10 @@
       <c r="Z12" s="8">
         <v>40.18452838575731</v>
       </c>
-      <c r="AA12" s="9">
-        <v>1</v>
-      </c>
-      <c r="AB12" s="9">
+      <c r="AA12" s="7">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="7">
         <v>1</v>
       </c>
       <c r="AC12" s="6" t="s">
@@ -2000,10 +2006,10 @@
       <c r="Z13" s="8">
         <v>26.88892750690754</v>
       </c>
-      <c r="AA13" s="9">
+      <c r="AA13" s="7">
         <v>6</v>
       </c>
-      <c r="AB13" s="9">
+      <c r="AB13" s="7">
         <v>2</v>
       </c>
       <c r="AC13" s="6" t="s">
@@ -2098,10 +2104,10 @@
       <c r="Z14" s="8">
         <v>30.74138453903112</v>
       </c>
-      <c r="AA14" s="9">
-        <v>2</v>
-      </c>
-      <c r="AB14" s="9">
+      <c r="AA14" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB14" s="7">
         <v>0</v>
       </c>
       <c r="AC14" s="6" t="s">
@@ -2412,7 +2418,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="9" t="s">
         <v>80</v>
       </c>
       <c r="B18" s="5">
@@ -2510,7 +2516,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="9" t="s">
         <v>83</v>
       </c>
       <c r="B19" s="5">
@@ -2608,7 +2614,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="17.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="10" t="s">
         <v>86</v>
       </c>
       <c r="B20" s="5">
@@ -2705,18 +2711,18 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="20.25">
-      <c r="A21" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
+      <c r="A21" s="11" t="s">
         <v>87</v>
       </c>
       <c r="B21" s="5">
-        <v>25568.875520833335</v>
+        <v>25568.375520833335</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E21" s="7">
         <v>167</v>
@@ -2728,67 +2734,67 @@
         <v>1.57</v>
       </c>
       <c r="H21" s="8">
-        <v>4.1</v>
+        <v>1</v>
       </c>
       <c r="I21" s="8">
-        <v>5.75</v>
+        <v>2</v>
       </c>
       <c r="J21" s="8">
-        <v>0.6038755619308649</v>
+        <v>3</v>
       </c>
       <c r="K21" s="8">
-        <v>0.2312401542027946</v>
+        <v>0.2554618627826753</v>
       </c>
       <c r="L21" s="8">
-        <v>0.1648842838663405</v>
+        <v>0.3049060942889996</v>
       </c>
       <c r="M21" s="8">
-        <v>0.05475815766188674</v>
+        <v>0.05796719450132803</v>
       </c>
       <c r="N21" s="7">
         <v>2</v>
       </c>
       <c r="O21" s="8">
-        <v>0.2068043869608158</v>
+        <v>0.3153639087876114</v>
       </c>
       <c r="P21" s="8">
-        <v>0.242857704879984</v>
+        <v>0.2454734549405155</v>
       </c>
       <c r="Q21" s="8">
-        <v>0.5503379081592003</v>
+        <v>0.4391626362718731</v>
       </c>
       <c r="R21" s="7">
         <v>1</v>
       </c>
       <c r="S21" s="8">
-        <v>0.3854536242928598</v>
+        <v>0.1342565419828735</v>
       </c>
       <c r="T21" s="7">
         <v>2</v>
       </c>
       <c r="U21" s="8">
-        <v>0.3854536242928598</v>
+        <v>0.1342565419828735</v>
       </c>
       <c r="V21" s="8">
-        <v>0.5503379081592003</v>
+        <v>0.4391626362718731</v>
       </c>
       <c r="W21" s="8">
-        <v>5.75</v>
+        <v>3.1</v>
       </c>
       <c r="X21" s="6" t="s">
         <v>44</v>
       </c>
       <c r="Y21" s="8">
-        <v>38.52365357114402</v>
+        <v>30.74138453903112</v>
       </c>
       <c r="Z21" s="8">
-        <v>38.52365357114402</v>
-      </c>
-      <c r="AA21" s="9">
-        <v>3</v>
-      </c>
-      <c r="AB21" s="9">
-        <v>2</v>
+        <v>30.74138453903112</v>
+      </c>
+      <c r="AA21" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB21" s="7">
+        <v>0</v>
       </c>
       <c r="AC21" s="6" t="s">
         <v>36</v>
@@ -2800,6 +2806,202 @@
         <v>1</v>
       </c>
       <c r="AF21" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="17.25">
+      <c r="A22" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" s="5">
+        <v>25568.375520833335</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E22" s="7">
+        <v>167</v>
+      </c>
+      <c r="F22" s="7">
+        <v>1671</v>
+      </c>
+      <c r="G22" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="H22" s="8">
+        <v>1</v>
+      </c>
+      <c r="I22" s="8">
+        <v>2</v>
+      </c>
+      <c r="J22" s="8">
+        <v>3</v>
+      </c>
+      <c r="K22" s="8">
+        <v>0.2554618627826753</v>
+      </c>
+      <c r="L22" s="8">
+        <v>0.3049060942889996</v>
+      </c>
+      <c r="M22" s="8">
+        <v>0.05796719450132803</v>
+      </c>
+      <c r="N22" s="7">
+        <v>2</v>
+      </c>
+      <c r="O22" s="8">
+        <v>0.3153639087876114</v>
+      </c>
+      <c r="P22" s="8">
+        <v>0.2454734549405155</v>
+      </c>
+      <c r="Q22" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="R22" s="7">
+        <v>1</v>
+      </c>
+      <c r="S22" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="T22" s="7">
+        <v>2</v>
+      </c>
+      <c r="U22" s="8">
+        <v>0.1342565419828735</v>
+      </c>
+      <c r="V22" s="8">
+        <v>0.4391626362718731</v>
+      </c>
+      <c r="W22" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="X22" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y22" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="Z22" s="8">
+        <v>30.74138453903112</v>
+      </c>
+      <c r="AA22" s="7">
+        <v>2</v>
+      </c>
+      <c r="AB22" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD22" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE22" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF22" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="20.25">
+      <c r="A23" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B23" s="5">
+        <v>25568.875520833335</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="E23" s="7">
+        <v>167</v>
+      </c>
+      <c r="F23" s="7">
+        <v>1671</v>
+      </c>
+      <c r="G23" s="8">
+        <v>1.57</v>
+      </c>
+      <c r="H23" s="8">
+        <v>4.1</v>
+      </c>
+      <c r="I23" s="8">
+        <v>5.75</v>
+      </c>
+      <c r="J23" s="8">
+        <v>0.6038755619308649</v>
+      </c>
+      <c r="K23" s="8">
+        <v>0.2312401542027946</v>
+      </c>
+      <c r="L23" s="8">
+        <v>0.1648842838663405</v>
+      </c>
+      <c r="M23" s="8">
+        <v>0.05475815766188674</v>
+      </c>
+      <c r="N23" s="7">
+        <v>2</v>
+      </c>
+      <c r="O23" s="8">
+        <v>0.2068043869608158</v>
+      </c>
+      <c r="P23" s="8">
+        <v>0.242857704879984</v>
+      </c>
+      <c r="Q23" s="8">
+        <v>0.5503379081592003</v>
+      </c>
+      <c r="R23" s="7">
+        <v>1</v>
+      </c>
+      <c r="S23" s="8">
+        <v>0.3854536242928598</v>
+      </c>
+      <c r="T23" s="7">
+        <v>2</v>
+      </c>
+      <c r="U23" s="8">
+        <v>0.3854536242928598</v>
+      </c>
+      <c r="V23" s="8">
+        <v>0.5503379081592003</v>
+      </c>
+      <c r="W23" s="8">
+        <v>5.75</v>
+      </c>
+      <c r="X23" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y23" s="8">
+        <v>38.52365357114402</v>
+      </c>
+      <c r="Z23" s="8">
+        <v>38.52365357114402</v>
+      </c>
+      <c r="AA23" s="7">
+        <v>3</v>
+      </c>
+      <c r="AB23" s="7">
+        <v>2</v>
+      </c>
+      <c r="AC23" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD23" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE23" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF23" s="7">
         <v>0</v>
       </c>
     </row>

</xml_diff>